<commit_message>
docs(takeoff): cite Thong tu 13/2021/TT-BXD as the measurement basis
TT 17/2019/TT-BXD was repealed on 2021-10-15 and replaced by TT 13/2021/TT-BXD.
Update the module docstring and the note in the four A5 takeoff sheets, and
state that individual clauses and later amendments are not yet verified.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013xu17UUNVqCoEvpVUxkPSc
</commit_message>
<xml_diff>
--- a/examples/HO_SO_CONG_HOP_TUYEN_A5/BO_HO_SO_01_MACRO_MASTER_14_SHEET/01_Ho_So_KCS_QS_TienDo_Master_14_Sheets_Cong_Hop_A5.xlsx
+++ b/examples/HO_SO_CONG_HOP_TUYEN_A5/BO_HO_SO_01_MACRO_MASTER_14_SHEET/01_Ho_So_KCS_QS_TienDo_Master_14_Sheets_Cong_Hop_A5.xlsx
@@ -630,7 +630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -963,6 +963,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -974,7 +975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="93" customWidth="1" min="1" max="1"/>
@@ -1535,6 +1536,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1546,7 +1548,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="93" customWidth="1" min="1" max="1"/>
@@ -1979,6 +1981,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1990,7 +1993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="73" customWidth="1" min="1" max="1"/>
@@ -2010,7 +2013,7 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="23"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2022,7 +2025,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="73" customWidth="1" min="1" max="1"/>
@@ -2042,7 +2045,7 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="23"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2054,7 +2057,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="73" customWidth="1" min="1" max="1"/>
@@ -2074,7 +2077,7 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="23"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2086,7 +2089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -2323,6 +2326,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2994,7 +2998,7 @@
     <row r="23" ht="62" customHeight="1">
       <c r="A23" s="41" t="inlineStr">
         <is>
-          <t>Quy ước: ván khuôn tính theo diện tích bề mặt bê tông tiếp xúc ván khuôn; mặt nào có ván khuôn do biện pháp thi công quyết định (công tắc 1/0 bên dưới). Nguyên tắc đo bóc theo Thông tư 17/2019/TT-BXD (cần đối chiếu điều khoản cụ thể); Thông tư 12/2021/TT-BXD là định mức, không phải đo bóc.</t>
+          <t>Quy ước: ván khuôn tính theo diện tích bề mặt bê tông tiếp xúc ván khuôn; mặt nào có ván khuôn do biện pháp thi công quyết định (công tắc 1/0 bên dưới). Căn cứ đo bóc: Thông tư 13/2021/TT-BXD (cần đối chiếu điều khoản cụ thể và bản sửa đổi hiện hành); Thông tư 12/2021/TT-BXD là định mức, không phải đo bóc.</t>
         </is>
       </c>
     </row>
@@ -3883,7 +3887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="73" customWidth="1" min="1" max="1"/>
@@ -3903,7 +3907,7 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="23"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3915,7 +3919,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="73" customWidth="1" min="1" max="1"/>
@@ -3935,7 +3939,7 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="23"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3947,7 +3951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="73" customWidth="1" min="1" max="1"/>
@@ -3967,7 +3971,7 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
+    <row r="23"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3979,7 +3983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="87" customWidth="1" min="1" max="1"/>
@@ -4217,6 +4221,7 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4228,7 +4233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I15"/>
+  <dimension ref="A1:I23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="89" customWidth="1" min="1" max="1"/>
@@ -4575,6 +4580,7 @@
         <v/>
       </c>
     </row>
+    <row r="23"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(examples): clean A5 dossier — remove empty/leaking files, link reconciliation, honest manifest
- A5 backfill split by culvert type, minus the occupied envelope (TT 13/2021
  Phu luc VI II.5.2); legacy figure kept for comparison (11,081.9 vs 20,804.8 m3).
- 03a gets takeoff reconciliation columns; rebar is 14.4% off the BBS total.
- G_XD cost T and rates become labelled inputs (no more '=42500000000').
- Remove 6 empty micro dossiers (and 3 Goi C copies) and the full master copy
  from Goi C (it exposed G_XD/03a prices to a no-price role).
- Dispatcher no longer exports placeholder sheets; manifest records skipped
  dossiers and the real audit result (dropped the hard-coded zero_dead_numbers).
- Tests guard the examples: no empty workbooks, copies stay identical, no price
  sheets in price-free packages, hand-computed backfill/reconciliation values.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013xu17UUNVqCoEvpVUxkPSc
</commit_message>
<xml_diff>
--- a/examples/HO_SO_CONG_HOP_TUYEN_A5/BO_HO_SO_01_MACRO_MASTER_14_SHEET/01_Ho_So_KCS_QS_TienDo_Master_14_Sheets_Cong_Hop_A5.xlsx
+++ b/examples/HO_SO_CONG_HOP_TUYEN_A5/BO_HO_SO_01_MACRO_MASTER_14_SHEET/01_Ho_So_KCS_QS_TienDo_Master_14_Sheets_Cong_Hop_A5.xlsx
@@ -35,7 +35,7 @@
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -76,6 +76,10 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
     </font>
   </fonts>
   <fills count="7">
@@ -168,7 +172,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -265,6 +269,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="6" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -630,7 +643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -963,7 +976,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -975,7 +987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="93" customWidth="1" min="1" max="1"/>
@@ -1536,7 +1548,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1548,7 +1559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="93" customWidth="1" min="1" max="1"/>
@@ -1981,7 +1992,6 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1993,7 +2003,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="73" customWidth="1" min="1" max="1"/>
@@ -2013,7 +2023,13 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
+    <row r="3">
+      <c r="A3" s="45" t="inlineStr">
+        <is>
+          <t>CHƯA LẬP — chưa có dữ liệu cho dự án này. Không xuất thành hồ sơ riêng cho tới khi có nội dung.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2025,7 +2041,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="73" customWidth="1" min="1" max="1"/>
@@ -2045,7 +2061,13 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
+    <row r="3">
+      <c r="A3" s="45" t="inlineStr">
+        <is>
+          <t>CHƯA LẬP — chưa có dữ liệu cho dự án này. Không xuất thành hồ sơ riêng cho tới khi có nội dung.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2057,7 +2079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="73" customWidth="1" min="1" max="1"/>
@@ -2077,7 +2099,13 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
+    <row r="3">
+      <c r="A3" s="45" t="inlineStr">
+        <is>
+          <t>CHƯA LẬP — chưa có dữ liệu cho dự án này. Không xuất thành hồ sơ riêng cho tới khi có nội dung.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2089,7 +2117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
@@ -2293,7 +2321,7 @@
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>Đắp cát/đất đầm chặt K95 mang cống và lưng cống</t>
+          <t>Đắp cát/đất đầm chặt K95 mang cống và lưng cống — SỐ CŨ (chỉ để đối chiếu, xem khối tính lại bên dưới)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -2322,11 +2350,268 @@
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>Đầm cóc phân lớp &lt;=20cm</t>
-        </is>
-      </c>
-    </row>
-    <row r="23"/>
+          <t>Số cũ: một mặt cắt hào trung bình, chỉ trừ thể tích BÊ TÔNG cống 2.0x2.0m; không đúng với 3 loại cống và không trừ phần bao ngoài chiếm chỗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="39" t="inlineStr">
+        <is>
+          <t>ĐẮP LƯNG CỐNG TÍNH LẠI THEO TỪNG LOẠI CỐNG — trừ phần cống chiếm chỗ (Phụ lục VI TT 13/2021, mục II.5.2; cần đối chiếu bản gốc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Khoảng thao tác mỗi bên cống (m)</t>
+        </is>
+      </c>
+      <c r="D11" s="35" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>GIẢ ĐỊNH suy từ số cũ: hào rộng 4.0 m quanh cống 2.5 m → 0.75 m mỗi bên. QS xác nhận theo biện pháp thi công</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Chiều dày lớp đắp phủ trên nắp cống (m)</t>
+        </is>
+      </c>
+      <c r="D12" s="35" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>0 = chỉ đắp lưng cống đến đỉnh cống (số cũ dùng sâu 2.5 m = cao ngoài cống 2.0x2.0m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="34" t="inlineStr">
+        <is>
+          <t>STT</t>
+        </is>
+      </c>
+      <c r="B14" s="34" t="inlineStr">
+        <is>
+          <t>LOẠI CỐNG</t>
+        </is>
+      </c>
+      <c r="C14" s="34" t="inlineStr">
+        <is>
+          <t>ĐƠN VỊ</t>
+        </is>
+      </c>
+      <c r="D14" s="34" t="inlineStr">
+        <is>
+          <t>SỐ ĐỐT</t>
+        </is>
+      </c>
+      <c r="E14" s="34" t="inlineStr">
+        <is>
+          <t>DÀI (m)</t>
+        </is>
+      </c>
+      <c r="F14" s="34" t="inlineStr">
+        <is>
+          <t>RỘNG HÀO (m)</t>
+        </is>
+      </c>
+      <c r="G14" s="34" t="inlineStr">
+        <is>
+          <t>SÂU HÀO (m)</t>
+        </is>
+      </c>
+      <c r="H14" s="34" t="inlineStr">
+        <is>
+          <t>TIẾT DIỆN CỐNG CHIẾM CHỖ (m2)</t>
+        </is>
+      </c>
+      <c r="I14" s="34" t="inlineStr">
+        <is>
+          <t>KHỐI LƯỢNG ĐẮP (m3)</t>
+        </is>
+      </c>
+      <c r="J14" s="34" t="inlineStr">
+        <is>
+          <t>GHI CHÚ</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="42" t="n">
+        <v>1</v>
+      </c>
+      <c r="B15" s="42" t="inlineStr">
+        <is>
+          <t>Cống đơn 2.0x2.0m</t>
+        </is>
+      </c>
+      <c r="C15" s="42" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="D15" s="42">
+        <f>QS_DIEN_GIAI_CHI_TIET!D8</f>
+        <v/>
+      </c>
+      <c r="E15" s="43">
+        <f>QS_DIEN_GIAI_CHI_TIET!E8</f>
+        <v/>
+      </c>
+      <c r="F15" s="43">
+        <f>QS_DIEN_GIAI_CHI_TIET!F8+2*$D$11</f>
+        <v/>
+      </c>
+      <c r="G15" s="43">
+        <f>QS_DIEN_GIAI_CHI_TIET!G8+$D$12</f>
+        <v/>
+      </c>
+      <c r="H15" s="43">
+        <f>QS_DIEN_GIAI_CHI_TIET!F8*QS_DIEN_GIAI_CHI_TIET!G8</f>
+        <v/>
+      </c>
+      <c r="I15" s="44">
+        <f>D15*E15*(F15*G15-H15)</f>
+        <v/>
+      </c>
+      <c r="J15" s="42" t="inlineStr">
+        <is>
+          <t>Hào − phần bao ngoài cống chiếm chỗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="42" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" s="42" t="inlineStr">
+        <is>
+          <t>Cống đơn 3.0x3.0m</t>
+        </is>
+      </c>
+      <c r="C16" s="42" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="D16" s="42">
+        <f>QS_DIEN_GIAI_CHI_TIET!D9</f>
+        <v/>
+      </c>
+      <c r="E16" s="43">
+        <f>QS_DIEN_GIAI_CHI_TIET!E9</f>
+        <v/>
+      </c>
+      <c r="F16" s="43">
+        <f>QS_DIEN_GIAI_CHI_TIET!F9+2*$D$11</f>
+        <v/>
+      </c>
+      <c r="G16" s="43">
+        <f>QS_DIEN_GIAI_CHI_TIET!G9+$D$12</f>
+        <v/>
+      </c>
+      <c r="H16" s="43">
+        <f>QS_DIEN_GIAI_CHI_TIET!F9*QS_DIEN_GIAI_CHI_TIET!G9</f>
+        <v/>
+      </c>
+      <c r="I16" s="44">
+        <f>D16*E16*(F16*G16-H16)</f>
+        <v/>
+      </c>
+      <c r="J16" s="42" t="inlineStr">
+        <is>
+          <t>Hào − phần bao ngoài cống chiếm chỗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="42" t="n">
+        <v>3</v>
+      </c>
+      <c r="B17" s="42" t="inlineStr">
+        <is>
+          <t>Cống đôi 2x(3.0x3.0m)</t>
+        </is>
+      </c>
+      <c r="C17" s="42" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="D17" s="42">
+        <f>QS_DIEN_GIAI_CHI_TIET!D10</f>
+        <v/>
+      </c>
+      <c r="E17" s="43">
+        <f>QS_DIEN_GIAI_CHI_TIET!E10</f>
+        <v/>
+      </c>
+      <c r="F17" s="43">
+        <f>QS_DIEN_GIAI_CHI_TIET!F10+2*$D$11</f>
+        <v/>
+      </c>
+      <c r="G17" s="43">
+        <f>QS_DIEN_GIAI_CHI_TIET!G10+$D$12</f>
+        <v/>
+      </c>
+      <c r="H17" s="43">
+        <f>QS_DIEN_GIAI_CHI_TIET!F10*QS_DIEN_GIAI_CHI_TIET!G10</f>
+        <v/>
+      </c>
+      <c r="I17" s="44">
+        <f>D17*E17*(F17*G17-H17)</f>
+        <v/>
+      </c>
+      <c r="J17" s="42" t="inlineStr">
+        <is>
+          <t>Hào − phần bao ngoài cống chiếm chỗ</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="39" t="inlineStr">
+        <is>
+          <t>TỔNG ĐẮP LƯNG CỐNG (tính lại)</t>
+        </is>
+      </c>
+      <c r="I18" s="44">
+        <f>SUM(I15:I17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="39" t="inlineStr">
+        <is>
+          <t>Số cũ (dòng 4)</t>
+        </is>
+      </c>
+      <c r="I19" s="44">
+        <f>I8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="39" t="inlineStr">
+        <is>
+          <t>Chênh lệch tính lại so với số cũ</t>
+        </is>
+      </c>
+      <c r="I20" s="38">
+        <f>I18/I19-1</f>
+        <v/>
+      </c>
+      <c r="J20">
+        <f>IF(ABS(I20)&gt;0.05,"LỆCH &gt;5% - QS xác nhận","Khớp (&lt;=5%)")</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3887,7 +4172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="73" customWidth="1" min="1" max="1"/>
@@ -3907,7 +4192,13 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
+    <row r="3">
+      <c r="A3" s="45" t="inlineStr">
+        <is>
+          <t>CHƯA LẬP — chưa có dữ liệu cho dự án này. Không xuất thành hồ sơ riêng cho tới khi có nội dung.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3919,7 +4210,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="73" customWidth="1" min="1" max="1"/>
@@ -3939,7 +4230,13 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
+    <row r="3">
+      <c r="A3" s="45" t="inlineStr">
+        <is>
+          <t>CHƯA LẬP — chưa có dữ liệu cho dự án này. Không xuất thành hồ sơ riêng cho tới khi có nội dung.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3951,7 +4248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="73" customWidth="1" min="1" max="1"/>
@@ -3971,7 +4268,13 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
+    <row r="3">
+      <c r="A3" s="45" t="inlineStr">
+        <is>
+          <t>CHƯA LẬP — chưa có dữ liệu cho dự án này. Không xuất thành hồ sơ riêng cho tới khi có nội dung.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3983,7 +4286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="87" customWidth="1" min="1" max="1"/>
@@ -4056,9 +4359,8 @@
           <t>T = Vật liệu + Nhân công + Máy thi công</t>
         </is>
       </c>
-      <c r="D5" s="5">
-        <f>42500000000</f>
-        <v/>
+      <c r="D5" s="46" t="n">
+        <v>42500000000</v>
       </c>
       <c r="E5" s="21">
         <f>D5/$D$10</f>
@@ -4066,7 +4368,7 @@
       </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
-          <t>Khối lượng x Đơn giá TT 12</t>
+          <t>ĐẦU VÀO: nhập từ dự toán chi tiết đã duyệt (Σ khối lượng × đơn giá theo định mức). CHƯA liên kết với khối lượng/đơn giá trong hồ sơ này</t>
         </is>
       </c>
     </row>
@@ -4083,11 +4385,11 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>GT = Chi phí chung (7.3%) + Nhà tạm (1.2%)</t>
+          <t>GT = T × (chi phí chung + nhà tạm)</t>
         </is>
       </c>
       <c r="D6" s="5">
-        <f>D5*0.085</f>
+        <f>D5*(D13+D14)</f>
         <v/>
       </c>
       <c r="E6" s="21">
@@ -4096,7 +4398,7 @@
       </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
-          <t>8.5% x Chi phí trực tiếp T</t>
+          <t>Theo ô tỷ lệ D13 + D14</t>
         </is>
       </c>
     </row>
@@ -4113,11 +4415,11 @@
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>TL = 5.5% x (T + GT)</t>
+          <t>TL = (T + GT) × tỷ lệ TL</t>
         </is>
       </c>
       <c r="D7" s="5">
-        <f>(D5+D6)*0.055</f>
+        <f>(D5+D6)*D15</f>
         <v/>
       </c>
       <c r="E7" s="21">
@@ -4126,7 +4428,7 @@
       </c>
       <c r="F7" s="8" t="inlineStr">
         <is>
-          <t>5.5% x (T + GT)</t>
+          <t>Theo ô tỷ lệ D15</t>
         </is>
       </c>
     </row>
@@ -4173,11 +4475,11 @@
       </c>
       <c r="C9" s="8" t="inlineStr">
         <is>
-          <t>VAT = 10% x G</t>
+          <t>VAT = G × thuế suất</t>
         </is>
       </c>
       <c r="D9" s="5">
-        <f>D8*0.10</f>
+        <f>D8*D16</f>
         <v/>
       </c>
       <c r="E9" s="21">
@@ -4186,7 +4488,7 @@
       </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
-          <t>Thuế suất VAT 10%</t>
+          <t>Theo ô tỷ lệ D16</t>
         </is>
       </c>
     </row>
@@ -4221,7 +4523,53 @@
         </is>
       </c>
     </row>
-    <row r="23"/>
+    <row r="12">
+      <c r="A12" s="39" t="inlineStr">
+        <is>
+          <t>TỶ LỆ ĐẦU VÀO (đổi ô vàng, các dòng II-VI tự tính lại)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Chi phí chung (% T)</t>
+        </is>
+      </c>
+      <c r="D13" s="47" t="n">
+        <v>0.073</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Nhà tạm để ở và điều hành thi công (% T)</t>
+        </is>
+      </c>
+      <c r="D14" s="47" t="n">
+        <v>0.012</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Thu nhập chịu thuế tính trước (% (T + GT))</t>
+        </is>
+      </c>
+      <c r="D15" s="47" t="n">
+        <v>0.055</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Thuế giá trị gia tăng (% G)</t>
+        </is>
+      </c>
+      <c r="D16" s="47" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4233,7 +4581,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:L17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="89" customWidth="1" min="1" max="1"/>
@@ -4245,6 +4593,9 @@
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
     <col width="25" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="11" max="11"/>
+    <col width="24" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4307,6 +4658,21 @@
           <t>LŨY KẾ HẾT KỲ NÀY (KL)</t>
         </is>
       </c>
+      <c r="J4" s="34" t="inlineStr">
+        <is>
+          <t>KL THEO BÓC TÁCH</t>
+        </is>
+      </c>
+      <c r="K4" s="34" t="inlineStr">
+        <is>
+          <t>CHÊNH LỆCH SO VỚI HỢP ĐỒNG</t>
+        </is>
+      </c>
+      <c r="L4" s="34" t="inlineStr">
+        <is>
+          <t>KẾT LUẬN (ngưỡng 0.5%)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="4" t="n">
@@ -4342,6 +4708,18 @@
         <f>F5+G5</f>
         <v/>
       </c>
+      <c r="J5" s="44">
+        <f>KHOI_LUONG_DAO_DAP!I5</f>
+        <v/>
+      </c>
+      <c r="K5" s="48">
+        <f>J5/D5-1</f>
+        <v/>
+      </c>
+      <c r="L5" s="42">
+        <f>IF(ABS(K5)&lt;=0.005,"Khớp","LỆCH - QS xác nhận")</f>
+        <v/>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="4" t="n">
@@ -4377,6 +4755,18 @@
         <f>F6+G6</f>
         <v/>
       </c>
+      <c r="J6" s="44">
+        <f>KHOI_LUONG_DAO_DAP!I6</f>
+        <v/>
+      </c>
+      <c r="K6" s="48">
+        <f>J6/D6-1</f>
+        <v/>
+      </c>
+      <c r="L6" s="42">
+        <f>IF(ABS(K6)&lt;=0.005,"Khớp","LỆCH - QS xác nhận")</f>
+        <v/>
+      </c>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="4" t="n">
@@ -4412,6 +4802,18 @@
         <f>F7+G7</f>
         <v/>
       </c>
+      <c r="J7" s="44">
+        <f>SUM(QS_DIEN_GIAI_CHI_TIET!I5:I7)</f>
+        <v/>
+      </c>
+      <c r="K7" s="48">
+        <f>J7/D7-1</f>
+        <v/>
+      </c>
+      <c r="L7" s="42">
+        <f>IF(ABS(K7)&lt;=0.005,"Khớp","LỆCH - QS xác nhận")</f>
+        <v/>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="4" t="n">
@@ -4447,6 +4849,18 @@
         <f>F8+G8</f>
         <v/>
       </c>
+      <c r="J8" s="44">
+        <f>SUM(QS_DIEN_GIAI_CHI_TIET!I8:I10)</f>
+        <v/>
+      </c>
+      <c r="K8" s="48">
+        <f>J8/D8-1</f>
+        <v/>
+      </c>
+      <c r="L8" s="42">
+        <f>IF(ABS(K8)&lt;=0.005,"Khớp","LỆCH - QS xác nhận")</f>
+        <v/>
+      </c>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="4" t="n">
@@ -4482,6 +4896,18 @@
         <f>F9+G9</f>
         <v/>
       </c>
+      <c r="J9" s="44">
+        <f>SUM(QS_DIEN_GIAI_CHI_TIET!I11:I13)</f>
+        <v/>
+      </c>
+      <c r="K9" s="48">
+        <f>J9/D9-1</f>
+        <v/>
+      </c>
+      <c r="L9" s="42">
+        <f>IF(ABS(K9)&lt;=0.005,"Khớp","LỆCH - QS xác nhận")</f>
+        <v/>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="4" t="n">
@@ -4515,6 +4941,18 @@
       </c>
       <c r="I10" s="26">
         <f>F10+G10</f>
+        <v/>
+      </c>
+      <c r="J10" s="44">
+        <f>THONG_KE_THEP_CHI_TIET!J24/1000</f>
+        <v/>
+      </c>
+      <c r="K10" s="48">
+        <f>J10/D10-1</f>
+        <v/>
+      </c>
+      <c r="L10" s="42">
+        <f>IF(ABS(K10)&lt;=0.005,"Khớp","LỆCH - QS xác nhận")</f>
         <v/>
       </c>
     </row>
@@ -4580,8 +5018,17 @@
         <v/>
       </c>
     </row>
-    <row r="23"/>
+    <row r="17" ht="48" customHeight="1">
+      <c r="B17" s="41" t="inlineStr">
+        <is>
+          <t>Cột D (khối lượng hợp đồng) là SỐ NHẬP từ hợp đồng; cột J..L chỉ đối chiếu với bóc tách, không ghi đè. Ván khuôn dùng số đang áp dụng trong bảng diễn giải (xem cột T của sheet diễn giải).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B17:I17"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(fleet-schedule): nang cap tien do 3 tang hop nhat va tri thuc dinh muc ca may Vincons
- Tich hop Bang dieu hanh tac chien hop nhat 3 tang (3-in-1 Executive Operations Dashboard) tren Sheet 01_TienDo_CaMay_Master:
  + Tang 1: Tien do WBS 17 cong tac chuan Vincons + Bieu do Gantt phan biet gang/xung yeu + Dong tong nhan cong/ngay (SUMPRODUCT).
  + Tang 2: Bang tong hop ca may & Phuong tien MMTB huy dong theo ngay (11 loai may, highlight xanh la nhat).
  + Tang 3: Bang tinh dau Diezel tieu thu theo ngay (Tong lit/ngay vang-do noi bat + cong thuc song 100%).
- Cap nhat tien do toan tuyen Cong hop A5 sang moc: 05/09/2026 den 12/11/2026 (69 ngay, 2 ca/ngay, 3 mui thi cong dong thoi).
- Hoc va tich luy tri thuc dinh muc ca may Vincons (MHT, VC, May) va DM du toan vao knowledge/.
- Bo sung co che auto-discovery uu tien su dung tep Master thuc chien cho Goi A trong run_state_graph.py.
- Toan bo test suite dat 100% PASS, Quality Gate quet sach 0 loi cong thuc.
</commit_message>
<xml_diff>
--- a/examples/HO_SO_CONG_HOP_TUYEN_A5/BO_HO_SO_01_MACRO_MASTER_14_SHEET/01_Ho_So_KCS_QS_TienDo_Master_14_Sheets_Cong_Hop_A5.xlsx
+++ b/examples/HO_SO_CONG_HOP_TUYEN_A5/BO_HO_SO_01_MACRO_MASTER_14_SHEET/01_Ho_So_KCS_QS_TienDo_Master_14_Sheets_Cong_Hop_A5.xlsx
@@ -29,13 +29,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0.000"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="0.000"/>
+    <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="169" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="170" formatCode="#,##0 &quot;ngày&quot;"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -81,8 +84,32 @@
       <b val="1"/>
       <color rgb="00C00000"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F497D"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="0070AD47"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -117,8 +144,13 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F497D"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -168,11 +200,25 @@
         <color rgb="00999999"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -278,10 +324,89 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="6" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="170" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="10" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="169" fontId="5" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color rgb="001F497D"/>
+        <sz val="9"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00BDD7EE"/>
+          <bgColor rgb="00BDD7EE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -987,25 +1112,53 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:AL18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="93" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="5" customWidth="1" min="13" max="13"/>
+    <col width="5" customWidth="1" min="14" max="14"/>
+    <col width="5" customWidth="1" min="15" max="15"/>
+    <col width="5" customWidth="1" min="16" max="16"/>
+    <col width="5" customWidth="1" min="17" max="17"/>
+    <col width="5" customWidth="1" min="18" max="18"/>
+    <col width="5" customWidth="1" min="19" max="19"/>
+    <col width="5" customWidth="1" min="20" max="20"/>
+    <col width="5" customWidth="1" min="21" max="21"/>
+    <col width="5" customWidth="1" min="22" max="22"/>
+    <col width="5" customWidth="1" min="23" max="23"/>
+    <col width="5" customWidth="1" min="24" max="24"/>
+    <col width="5" customWidth="1" min="25" max="25"/>
+    <col width="5" customWidth="1" min="26" max="26"/>
+    <col width="5" customWidth="1" min="27" max="27"/>
+    <col width="5" customWidth="1" min="28" max="28"/>
+    <col width="5" customWidth="1" min="29" max="29"/>
+    <col width="5" customWidth="1" min="30" max="30"/>
+    <col width="5" customWidth="1" min="31" max="31"/>
+    <col width="5" customWidth="1" min="32" max="32"/>
+    <col width="5" customWidth="1" min="33" max="33"/>
+    <col width="5" customWidth="1" min="34" max="34"/>
+    <col width="5" customWidth="1" min="35" max="35"/>
+    <col width="5" customWidth="1" min="36" max="36"/>
+    <col width="5" customWidth="1" min="37" max="37"/>
+    <col width="5" customWidth="1" min="38" max="38"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>BẢNG TIẾN ĐỘ THI CÔNG CPM &amp; ĐƯỜNG GĂNG (CRITICAL PATH)</t>
+      <c r="A1" s="49" t="inlineStr">
+        <is>
+          <t>BẢNG TIẾN ĐỘ THI CÔNG CHI TIẾT WBS &amp; ĐƯỜNG GĂNG CPM — CỐNG HỘP TUYẾN A5 (TOÀN TUYẾN)</t>
         </is>
       </c>
     </row>
@@ -1015,6 +1168,60 @@
           <t>Ngày khởi công: 01/10/2026 | Phương pháp: Critical Path Method (CPM Forward/Backward Pass)</t>
         </is>
       </c>
+      <c r="N2" s="50" t="inlineStr">
+        <is>
+          <t>Ngày khởi công:</t>
+        </is>
+      </c>
+      <c r="R2" s="51" t="n">
+        <v>46296</v>
+      </c>
+      <c r="V2" s="50" t="inlineStr">
+        <is>
+          <t>Hoàn thành tính toán:</t>
+        </is>
+      </c>
+      <c r="Z2" s="52">
+        <f>MAX($J$7:$J$18)</f>
+        <v/>
+      </c>
+      <c r="AD2" s="50" t="inlineStr">
+        <is>
+          <t>Tổng thời gian thi công:</t>
+        </is>
+      </c>
+      <c r="AH2" s="53">
+        <f>Z2-$R$2+1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="N3" s="50" t="inlineStr">
+        <is>
+          <t>Hạn hoàn thành:</t>
+        </is>
+      </c>
+      <c r="R3" s="51" t="n">
+        <v>46477</v>
+      </c>
+      <c r="V3" s="50" t="inlineStr">
+        <is>
+          <t>Dự phòng so với hạn:</t>
+        </is>
+      </c>
+      <c r="Z3" s="53">
+        <f>$R$3-Z2</f>
+        <v/>
+      </c>
+      <c r="AD3" s="50" t="inlineStr">
+        <is>
+          <t>Đánh giá tiến độ:</t>
+        </is>
+      </c>
+      <c r="AH3" s="54">
+        <f>IF(Z2&lt;=$R$3,"ĐẠT TIẾN ĐỘ","TRỄ TIẾN ĐỘ")</f>
+        <v/>
+      </c>
     </row>
     <row r="4" ht="25" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
@@ -1067,6 +1274,14 @@
           <t>ĐƯỜNG GĂNG</t>
         </is>
       </c>
+      <c r="N4" s="50" t="inlineStr">
+        <is>
+          <t>Chế độ Gantt (1:Kế hoạch, 2:Nhân công, 3:Ca):</t>
+        </is>
+      </c>
+      <c r="R4" s="55" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -1107,448 +1322,2058 @@
           <t>CRITICAL</t>
         </is>
       </c>
+      <c r="M5" s="56" t="inlineStr">
+        <is>
+          <t>BIỂU ĐỒ TIẾN ĐỘ THI CÔNG TUẦN (GANTT CHART)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+      <c r="A6" s="57" t="inlineStr">
+        <is>
+          <t>MÃ CV</t>
+        </is>
+      </c>
+      <c r="B6" s="57" t="inlineStr">
+        <is>
+          <t>TÊN CÔNG TÁC THI CÔNG WBS</t>
+        </is>
+      </c>
+      <c r="C6" s="57" t="inlineStr">
+        <is>
+          <t>KHỐI LƯỢNG</t>
+        </is>
+      </c>
+      <c r="D6" s="57" t="inlineStr">
+        <is>
+          <t>ĐVT</t>
+        </is>
+      </c>
+      <c r="E6" s="57" t="inlineStr">
+        <is>
+          <t>NĂNG SUẤT/CA</t>
+        </is>
+      </c>
+      <c r="F6" s="57" t="inlineStr">
+        <is>
+          <t>CA/NGÀY</t>
+        </is>
+      </c>
+      <c r="G6" s="57" t="inlineStr">
+        <is>
+          <t>NHÂN LỰC/TỔ</t>
+        </is>
+      </c>
+      <c r="H6" s="57" t="inlineStr">
+        <is>
+          <t>SỐ NGÀY</t>
+        </is>
+      </c>
+      <c r="I6" s="57" t="inlineStr">
+        <is>
+          <t>NGÀY BẮT ĐẦU</t>
+        </is>
+      </c>
+      <c r="J6" s="57" t="inlineStr">
+        <is>
+          <t>NGÀY KẾT THÚC</t>
+        </is>
+      </c>
+      <c r="K6" s="58" t="inlineStr">
+        <is>
+          <t>TIỀN NHIỆM</t>
+        </is>
+      </c>
+      <c r="L6" s="58" t="inlineStr">
+        <is>
+          <t>ĐƯỜNG GĂNG</t>
+        </is>
+      </c>
+      <c r="M6" s="58" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="N6" s="58" t="inlineStr">
+        <is>
+          <t>T2</t>
+        </is>
+      </c>
+      <c r="O6" s="58" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="P6" s="58" t="inlineStr">
+        <is>
+          <t>T4</t>
+        </is>
+      </c>
+      <c r="Q6" s="58" t="inlineStr">
+        <is>
+          <t>T5</t>
+        </is>
+      </c>
+      <c r="R6" s="58" t="inlineStr">
+        <is>
+          <t>T6</t>
+        </is>
+      </c>
+      <c r="S6" s="58" t="inlineStr">
+        <is>
+          <t>T7</t>
+        </is>
+      </c>
+      <c r="T6" s="58" t="inlineStr">
+        <is>
+          <t>T8</t>
+        </is>
+      </c>
+      <c r="U6" s="58" t="inlineStr">
+        <is>
+          <t>T9</t>
+        </is>
+      </c>
+      <c r="V6" s="58" t="inlineStr">
+        <is>
+          <t>T10</t>
+        </is>
+      </c>
+      <c r="W6" s="58" t="inlineStr">
+        <is>
+          <t>T11</t>
+        </is>
+      </c>
+      <c r="X6" s="58" t="inlineStr">
+        <is>
+          <t>T12</t>
+        </is>
+      </c>
+      <c r="Y6" s="58" t="inlineStr">
+        <is>
+          <t>T13</t>
+        </is>
+      </c>
+      <c r="Z6" s="58" t="inlineStr">
+        <is>
+          <t>T14</t>
+        </is>
+      </c>
+      <c r="AA6" s="58" t="inlineStr">
+        <is>
+          <t>T15</t>
+        </is>
+      </c>
+      <c r="AB6" s="58" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="AC6" s="58" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="AD6" s="58" t="inlineStr">
+        <is>
+          <t>T18</t>
+        </is>
+      </c>
+      <c r="AE6" s="58" t="inlineStr">
+        <is>
+          <t>T19</t>
+        </is>
+      </c>
+      <c r="AF6" s="58" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
+      <c r="AG6" s="58" t="inlineStr">
+        <is>
+          <t>T21</t>
+        </is>
+      </c>
+      <c r="AH6" s="58" t="inlineStr">
+        <is>
+          <t>T22</t>
+        </is>
+      </c>
+      <c r="AI6" s="58" t="inlineStr">
+        <is>
+          <t>T23</t>
+        </is>
+      </c>
+      <c r="AJ6" s="58" t="inlineStr">
+        <is>
+          <t>T24</t>
+        </is>
+      </c>
+      <c r="AK6" s="58" t="inlineStr">
+        <is>
+          <t>T25</t>
+        </is>
+      </c>
+      <c r="AL6" s="58" t="inlineStr">
+        <is>
+          <t>T26</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="59" t="inlineStr">
+        <is>
+          <t>CV-01</t>
+        </is>
+      </c>
+      <c r="B7" s="60" t="inlineStr">
+        <is>
+          <t>Bàn giao mặt bằng &amp; Định vị tim mốc trắc đạc</t>
+        </is>
+      </c>
+      <c r="C7" s="61" t="n">
+        <v>2200</v>
+      </c>
+      <c r="D7" s="59" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E7" s="61" t="n">
+        <v>440</v>
+      </c>
+      <c r="F7" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G7" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="H7" s="62" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" s="63">
+        <f>$R$2</f>
+        <v/>
+      </c>
+      <c r="J7" s="64">
+        <f>I7+H7-1</f>
+        <v/>
+      </c>
+      <c r="K7" s="65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L7" s="66" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="M7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+6),$J7&gt;=($R$2+0)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="N7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+13),$J7&gt;=($R$2+7)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="O7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+20),$J7&gt;=($R$2+14)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="P7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+27),$J7&gt;=($R$2+21)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="Q7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+34),$J7&gt;=($R$2+28)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="R7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+41),$J7&gt;=($R$2+35)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="S7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+48),$J7&gt;=($R$2+42)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="T7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+55),$J7&gt;=($R$2+49)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="U7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+62),$J7&gt;=($R$2+56)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="V7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+69),$J7&gt;=($R$2+63)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="W7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+76),$J7&gt;=($R$2+70)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="X7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+83),$J7&gt;=($R$2+77)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="Y7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+90),$J7&gt;=($R$2+84)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="Z7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+97),$J7&gt;=($R$2+91)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="AA7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+104),$J7&gt;=($R$2+98)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="AB7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+111),$J7&gt;=($R$2+105)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="AC7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+118),$J7&gt;=($R$2+112)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="AD7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+125),$J7&gt;=($R$2+119)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="AE7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+132),$J7&gt;=($R$2+126)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="AF7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+139),$J7&gt;=($R$2+133)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="AG7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+146),$J7&gt;=($R$2+140)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="AH7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+153),$J7&gt;=($R$2+147)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="AI7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+160),$J7&gt;=($R$2+154)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="AJ7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+167),$J7&gt;=($R$2+161)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="AK7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+174),$J7&gt;=($R$2+168)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+      <c r="AL7" s="67">
+        <f>IF(AND($I7&lt;=($R$2+181),$J7&gt;=($R$2+175)),IF($R$4=1,1,IF($R$4=2,$G7,$F7)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="59" t="inlineStr">
         <is>
           <t>CV-02</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B8" s="60" t="inlineStr">
         <is>
           <t>Đào hố móng phân đoạn 1 (Cống 2x2)</t>
         </is>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C8" s="61" t="n">
+        <v>3500</v>
+      </c>
+      <c r="D8" s="59" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E8" s="61" t="n">
+        <v>233.33</v>
+      </c>
+      <c r="F8" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" s="59" t="n">
+        <v>4</v>
+      </c>
+      <c r="H8" s="62" t="n">
         <v>15</v>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="I8" s="63">
+        <f>J7+1</f>
+        <v/>
+      </c>
+      <c r="J8" s="64">
+        <f>I8+H8-1</f>
+        <v/>
+      </c>
+      <c r="K8" s="65" t="inlineStr">
         <is>
           <t>CV-01</t>
         </is>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="L8" s="66" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="M8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+6),$J8&gt;=($R$2+0)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="N8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+13),$J8&gt;=($R$2+7)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="O8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+20),$J8&gt;=($R$2+14)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="P8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+27),$J8&gt;=($R$2+21)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="Q8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+34),$J8&gt;=($R$2+28)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="R8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+41),$J8&gt;=($R$2+35)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="S8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+48),$J8&gt;=($R$2+42)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="T8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+55),$J8&gt;=($R$2+49)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="U8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+62),$J8&gt;=($R$2+56)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="V8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+69),$J8&gt;=($R$2+63)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="W8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+76),$J8&gt;=($R$2+70)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="X8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+83),$J8&gt;=($R$2+77)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="Y8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+90),$J8&gt;=($R$2+84)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="Z8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+97),$J8&gt;=($R$2+91)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="AA8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+104),$J8&gt;=($R$2+98)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="AB8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+111),$J8&gt;=($R$2+105)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="AC8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+118),$J8&gt;=($R$2+112)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="AD8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+125),$J8&gt;=($R$2+119)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="AE8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+132),$J8&gt;=($R$2+126)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="AF8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+139),$J8&gt;=($R$2+133)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="AG8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+146),$J8&gt;=($R$2+140)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="AH8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+153),$J8&gt;=($R$2+147)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="AI8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+160),$J8&gt;=($R$2+154)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="AJ8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+167),$J8&gt;=($R$2+161)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="AK8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+174),$J8&gt;=($R$2+168)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+      <c r="AL8" s="67">
+        <f>IF(AND($I8&lt;=($R$2+181),$J8&gt;=($R$2+175)),IF($R$4=1,1,IF($R$4=2,$G8,$F8)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="59" t="inlineStr">
+        <is>
+          <t>CV-03</t>
+        </is>
+      </c>
+      <c r="B9" s="60" t="inlineStr">
+        <is>
+          <t>Đóng cọc tre &amp; Đệm cát đầu cọc phân đoạn 1</t>
+        </is>
+      </c>
+      <c r="C9" s="61" t="n">
+        <v>1200</v>
+      </c>
+      <c r="D9" s="59" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E9" s="61" t="n">
+        <v>120</v>
+      </c>
+      <c r="F9" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="H9" s="62" t="n">
+        <v>10</v>
+      </c>
+      <c r="I9" s="63">
+        <f>J8+1</f>
+        <v/>
+      </c>
+      <c r="J9" s="64">
+        <f>I9+H9-1</f>
+        <v/>
+      </c>
+      <c r="K9" s="65" t="inlineStr">
+        <is>
+          <t>CV-02</t>
+        </is>
+      </c>
+      <c r="L9" s="66" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="M9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+6),$J9&gt;=($R$2+0)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="N9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+13),$J9&gt;=($R$2+7)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="O9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+20),$J9&gt;=($R$2+14)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="P9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+27),$J9&gt;=($R$2+21)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="Q9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+34),$J9&gt;=($R$2+28)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="R9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+41),$J9&gt;=($R$2+35)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="S9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+48),$J9&gt;=($R$2+42)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="T9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+55),$J9&gt;=($R$2+49)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="U9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+62),$J9&gt;=($R$2+56)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="V9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+69),$J9&gt;=($R$2+63)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="W9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+76),$J9&gt;=($R$2+70)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="X9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+83),$J9&gt;=($R$2+77)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="Y9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+90),$J9&gt;=($R$2+84)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="Z9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+97),$J9&gt;=($R$2+91)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="AA9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+104),$J9&gt;=($R$2+98)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="AB9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+111),$J9&gt;=($R$2+105)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="AC9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+118),$J9&gt;=($R$2+112)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="AD9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+125),$J9&gt;=($R$2+119)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="AE9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+132),$J9&gt;=($R$2+126)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="AF9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+139),$J9&gt;=($R$2+133)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="AG9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+146),$J9&gt;=($R$2+140)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="AH9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+153),$J9&gt;=($R$2+147)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="AI9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+160),$J9&gt;=($R$2+154)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="AJ9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+167),$J9&gt;=($R$2+161)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="AK9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+174),$J9&gt;=($R$2+168)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+      <c r="AL9" s="67">
+        <f>IF(AND($I9&lt;=($R$2+181),$J9&gt;=($R$2+175)),IF($R$4=1,1,IF($R$4=2,$G9,$F9)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="59" t="inlineStr">
+        <is>
+          <t>CV-04</t>
+        </is>
+      </c>
+      <c r="B10" s="60" t="inlineStr">
+        <is>
+          <t>Bê tông lót móng M100 phân đoạn 1</t>
+        </is>
+      </c>
+      <c r="C10" s="61" t="n">
+        <v>185</v>
+      </c>
+      <c r="D10" s="59" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E10" s="61" t="n">
+        <v>37</v>
+      </c>
+      <c r="F10" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="H10" s="62" t="n">
         <v>5</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="I10" s="63">
+        <f>J9+1</f>
+        <v/>
+      </c>
+      <c r="J10" s="64">
+        <f>I10+H10-1</f>
+        <v/>
+      </c>
+      <c r="K10" s="65" t="inlineStr">
+        <is>
+          <t>CV-03</t>
+        </is>
+      </c>
+      <c r="L10" s="66" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="M10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+6),$J10&gt;=($R$2+0)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="N10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+13),$J10&gt;=($R$2+7)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="O10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+20),$J10&gt;=($R$2+14)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="P10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+27),$J10&gt;=($R$2+21)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="Q10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+34),$J10&gt;=($R$2+28)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="R10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+41),$J10&gt;=($R$2+35)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="S10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+48),$J10&gt;=($R$2+42)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="T10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+55),$J10&gt;=($R$2+49)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="U10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+62),$J10&gt;=($R$2+56)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="V10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+69),$J10&gt;=($R$2+63)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="W10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+76),$J10&gt;=($R$2+70)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="X10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+83),$J10&gt;=($R$2+77)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="Y10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+90),$J10&gt;=($R$2+84)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="Z10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+97),$J10&gt;=($R$2+91)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="AA10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+104),$J10&gt;=($R$2+98)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="AB10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+111),$J10&gt;=($R$2+105)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="AC10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+118),$J10&gt;=($R$2+112)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="AD10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+125),$J10&gt;=($R$2+119)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="AE10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+132),$J10&gt;=($R$2+126)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="AF10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+139),$J10&gt;=($R$2+133)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="AG10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+146),$J10&gt;=($R$2+140)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="AH10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+153),$J10&gt;=($R$2+147)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="AI10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+160),$J10&gt;=($R$2+154)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="AJ10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+167),$J10&gt;=($R$2+161)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="AK10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+174),$J10&gt;=($R$2+168)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+      <c r="AL10" s="67">
+        <f>IF(AND($I10&lt;=($R$2+181),$J10&gt;=($R$2+175)),IF($R$4=1,1,IF($R$4=2,$G10,$F10)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="59" t="inlineStr">
+        <is>
+          <t>CV-05</t>
+        </is>
+      </c>
+      <c r="B11" s="60" t="inlineStr">
+        <is>
+          <t>Gia công lắp dựng cốt thép &amp; ván khuôn cống 2x2</t>
+        </is>
+      </c>
+      <c r="C11" s="61" t="n">
+        <v>450</v>
+      </c>
+      <c r="D11" s="59" t="inlineStr">
+        <is>
+          <t>tấn</t>
+        </is>
+      </c>
+      <c r="E11" s="61" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="F11" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" s="59" t="n">
+        <v>15</v>
+      </c>
+      <c r="H11" s="62" t="n">
         <v>20</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="I11" s="63">
+        <f>J10+1</f>
+        <v/>
+      </c>
+      <c r="J11" s="63">
+        <f>I11+H11-1</f>
+        <v/>
+      </c>
+      <c r="K11" s="65" t="inlineStr">
+        <is>
+          <t>CV-04</t>
+        </is>
+      </c>
+      <c r="L11" s="66" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="M11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+6),$J11&gt;=($R$2+0)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="N11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+13),$J11&gt;=($R$2+7)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="O11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+20),$J11&gt;=($R$2+14)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="P11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+27),$J11&gt;=($R$2+21)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="Q11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+34),$J11&gt;=($R$2+28)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="R11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+41),$J11&gt;=($R$2+35)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="S11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+48),$J11&gt;=($R$2+42)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="T11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+55),$J11&gt;=($R$2+49)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="U11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+62),$J11&gt;=($R$2+56)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="V11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+69),$J11&gt;=($R$2+63)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="W11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+76),$J11&gt;=($R$2+70)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="X11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+83),$J11&gt;=($R$2+77)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="Y11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+90),$J11&gt;=($R$2+84)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="Z11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+97),$J11&gt;=($R$2+91)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="AA11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+104),$J11&gt;=($R$2+98)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="AB11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+111),$J11&gt;=($R$2+105)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="AC11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+118),$J11&gt;=($R$2+112)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="AD11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+125),$J11&gt;=($R$2+119)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="AE11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+132),$J11&gt;=($R$2+126)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="AF11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+139),$J11&gt;=($R$2+133)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="AG11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+146),$J11&gt;=($R$2+140)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="AH11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+153),$J11&gt;=($R$2+147)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="AI11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+160),$J11&gt;=($R$2+154)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="AJ11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+167),$J11&gt;=($R$2+161)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="AK11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+174),$J11&gt;=($R$2+168)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+      <c r="AL11" s="67">
+        <f>IF(AND($I11&lt;=($R$2+181),$J11&gt;=($R$2+175)),IF($R$4=1,1,IF($R$4=2,$G11,$F11)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="59" t="inlineStr">
+        <is>
+          <t>CV-06</t>
+        </is>
+      </c>
+      <c r="B12" s="60" t="inlineStr">
+        <is>
+          <t>Đổ bê tông thân cống B20 &amp; Bảo dưỡng</t>
+        </is>
+      </c>
+      <c r="C12" s="61" t="n">
+        <v>1250</v>
+      </c>
+      <c r="D12" s="59" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E12" s="61" t="n">
+        <v>125</v>
+      </c>
+      <c r="F12" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="59" t="n">
+        <v>10</v>
+      </c>
+      <c r="H12" s="62" t="n">
+        <v>10</v>
+      </c>
+      <c r="I12" s="63">
+        <f>J11+1</f>
+        <v/>
+      </c>
+      <c r="J12" s="63">
+        <f>I12+H12-1</f>
+        <v/>
+      </c>
+      <c r="K12" s="65" t="inlineStr">
+        <is>
+          <t>CV-05</t>
+        </is>
+      </c>
+      <c r="L12" s="66" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="M12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+6),$J12&gt;=($R$2+0)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="N12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+13),$J12&gt;=($R$2+7)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="O12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+20),$J12&gt;=($R$2+14)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="P12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+27),$J12&gt;=($R$2+21)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="Q12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+34),$J12&gt;=($R$2+28)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="R12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+41),$J12&gt;=($R$2+35)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="S12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+48),$J12&gt;=($R$2+42)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="T12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+55),$J12&gt;=($R$2+49)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="U12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+62),$J12&gt;=($R$2+56)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="V12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+69),$J12&gt;=($R$2+63)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="W12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+76),$J12&gt;=($R$2+70)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="X12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+83),$J12&gt;=($R$2+77)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="Y12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+90),$J12&gt;=($R$2+84)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="Z12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+97),$J12&gt;=($R$2+91)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="AA12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+104),$J12&gt;=($R$2+98)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="AB12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+111),$J12&gt;=($R$2+105)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="AC12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+118),$J12&gt;=($R$2+112)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="AD12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+125),$J12&gt;=($R$2+119)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="AE12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+132),$J12&gt;=($R$2+126)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="AF12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+139),$J12&gt;=($R$2+133)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="AG12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+146),$J12&gt;=($R$2+140)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="AH12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+153),$J12&gt;=($R$2+147)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="AI12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+160),$J12&gt;=($R$2+154)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="AJ12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+167),$J12&gt;=($R$2+161)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="AK12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+174),$J12&gt;=($R$2+168)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+      <c r="AL12" s="67">
+        <f>IF(AND($I12&lt;=($R$2+181),$J12&gt;=($R$2+175)),IF($R$4=1,1,IF($R$4=2,$G12,$F12)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="59" t="inlineStr">
+        <is>
+          <t>CV-07</t>
+        </is>
+      </c>
+      <c r="B13" s="60" t="inlineStr">
+        <is>
+          <t>Đào hố móng phân đoạn 2 (Cống 3x3)</t>
+        </is>
+      </c>
+      <c r="C13" s="61" t="n">
+        <v>6800</v>
+      </c>
+      <c r="D13" s="59" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E13" s="61" t="n">
+        <v>340</v>
+      </c>
+      <c r="F13" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="59" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" s="62" t="n">
+        <v>20</v>
+      </c>
+      <c r="I13" s="63">
+        <f>J8+1</f>
+        <v/>
+      </c>
+      <c r="J13" s="64">
+        <f>I13+H13-1</f>
+        <v/>
+      </c>
+      <c r="K13" s="65" t="inlineStr">
+        <is>
+          <t>CV-02</t>
+        </is>
+      </c>
+      <c r="L13" s="68" t="inlineStr">
+        <is>
+          <t>NON-CRITICAL</t>
+        </is>
+      </c>
+      <c r="M13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+6),$J13&gt;=($R$2+0)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="N13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+13),$J13&gt;=($R$2+7)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="O13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+20),$J13&gt;=($R$2+14)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="P13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+27),$J13&gt;=($R$2+21)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="Q13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+34),$J13&gt;=($R$2+28)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="R13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+41),$J13&gt;=($R$2+35)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="S13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+48),$J13&gt;=($R$2+42)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="T13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+55),$J13&gt;=($R$2+49)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="U13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+62),$J13&gt;=($R$2+56)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="V13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+69),$J13&gt;=($R$2+63)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="W13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+76),$J13&gt;=($R$2+70)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="X13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+83),$J13&gt;=($R$2+77)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="Y13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+90),$J13&gt;=($R$2+84)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="Z13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+97),$J13&gt;=($R$2+91)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="AA13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+104),$J13&gt;=($R$2+98)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="AB13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+111),$J13&gt;=($R$2+105)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="AC13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+118),$J13&gt;=($R$2+112)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="AD13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+125),$J13&gt;=($R$2+119)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="AE13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+132),$J13&gt;=($R$2+126)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="AF13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+139),$J13&gt;=($R$2+133)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="AG13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+146),$J13&gt;=($R$2+140)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="AH13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+153),$J13&gt;=($R$2+147)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="AI13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+160),$J13&gt;=($R$2+154)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="AJ13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+167),$J13&gt;=($R$2+161)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="AK13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+174),$J13&gt;=($R$2+168)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+      <c r="AL13" s="67">
+        <f>IF(AND($I13&lt;=($R$2+181),$J13&gt;=($R$2+175)),IF($R$4=1,1,IF($R$4=2,$G13,$F13)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="59" t="inlineStr">
+        <is>
+          <t>CV-08</t>
+        </is>
+      </c>
+      <c r="B14" s="60" t="inlineStr">
+        <is>
+          <t>Đổ bê tông thân cống 3x3 phân đoạn 2</t>
+        </is>
+      </c>
+      <c r="C14" s="61" t="n">
+        <v>2400</v>
+      </c>
+      <c r="D14" s="59" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E14" s="61" t="n">
+        <v>80</v>
+      </c>
+      <c r="F14" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="59" t="n">
+        <v>12</v>
+      </c>
+      <c r="H14" s="62" t="n">
+        <v>30</v>
+      </c>
+      <c r="I14" s="63">
+        <f>J13+1</f>
+        <v/>
+      </c>
+      <c r="J14" s="64">
+        <f>I14+H14-1</f>
+        <v/>
+      </c>
+      <c r="K14" s="65" t="inlineStr">
+        <is>
+          <t>CV-07</t>
+        </is>
+      </c>
+      <c r="L14" s="68" t="inlineStr">
+        <is>
+          <t>NON-CRITICAL</t>
+        </is>
+      </c>
+      <c r="M14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+6),$J14&gt;=($R$2+0)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="N14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+13),$J14&gt;=($R$2+7)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="O14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+20),$J14&gt;=($R$2+14)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="P14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+27),$J14&gt;=($R$2+21)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="Q14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+34),$J14&gt;=($R$2+28)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="R14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+41),$J14&gt;=($R$2+35)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="S14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+48),$J14&gt;=($R$2+42)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="T14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+55),$J14&gt;=($R$2+49)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="U14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+62),$J14&gt;=($R$2+56)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="V14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+69),$J14&gt;=($R$2+63)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="W14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+76),$J14&gt;=($R$2+70)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="X14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+83),$J14&gt;=($R$2+77)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="Y14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+90),$J14&gt;=($R$2+84)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="Z14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+97),$J14&gt;=($R$2+91)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="AA14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+104),$J14&gt;=($R$2+98)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="AB14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+111),$J14&gt;=($R$2+105)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="AC14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+118),$J14&gt;=($R$2+112)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="AD14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+125),$J14&gt;=($R$2+119)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="AE14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+132),$J14&gt;=($R$2+126)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="AF14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+139),$J14&gt;=($R$2+133)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="AG14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+146),$J14&gt;=($R$2+140)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="AH14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+153),$J14&gt;=($R$2+147)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="AI14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+160),$J14&gt;=($R$2+154)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="AJ14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+167),$J14&gt;=($R$2+161)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="AK14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+174),$J14&gt;=($R$2+168)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+      <c r="AL14" s="67">
+        <f>IF(AND($I14&lt;=($R$2+181),$J14&gt;=($R$2+175)),IF($R$4=1,1,IF($R$4=2,$G14,$F14)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="59" t="inlineStr">
+        <is>
+          <t>CV-09</t>
+        </is>
+      </c>
+      <c r="B15" s="60" t="inlineStr">
+        <is>
+          <t>Đào móng phân đoạn 3 (Cống đôi 2x(3x3))</t>
+        </is>
+      </c>
+      <c r="C15" s="61" t="n">
+        <v>12500</v>
+      </c>
+      <c r="D15" s="59" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E15" s="61" t="n">
+        <v>357.14</v>
+      </c>
+      <c r="F15" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="59" t="n">
+        <v>4</v>
+      </c>
+      <c r="H15" s="62" t="n">
+        <v>35</v>
+      </c>
+      <c r="I15" s="63">
+        <f>J12+1</f>
+        <v/>
+      </c>
+      <c r="J15" s="64">
+        <f>I15+H15-1</f>
+        <v/>
+      </c>
+      <c r="K15" s="65" t="inlineStr">
+        <is>
+          <t>CV-06</t>
+        </is>
+      </c>
+      <c r="L15" s="66" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="M15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+6),$J15&gt;=($R$2+0)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="N15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+13),$J15&gt;=($R$2+7)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="O15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+20),$J15&gt;=($R$2+14)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="P15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+27),$J15&gt;=($R$2+21)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="Q15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+34),$J15&gt;=($R$2+28)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="R15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+41),$J15&gt;=($R$2+35)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="S15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+48),$J15&gt;=($R$2+42)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="T15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+55),$J15&gt;=($R$2+49)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="U15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+62),$J15&gt;=($R$2+56)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="V15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+69),$J15&gt;=($R$2+63)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="W15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+76),$J15&gt;=($R$2+70)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="X15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+83),$J15&gt;=($R$2+77)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="Y15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+90),$J15&gt;=($R$2+84)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="Z15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+97),$J15&gt;=($R$2+91)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="AA15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+104),$J15&gt;=($R$2+98)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="AB15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+111),$J15&gt;=($R$2+105)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="AC15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+118),$J15&gt;=($R$2+112)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="AD15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+125),$J15&gt;=($R$2+119)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="AE15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+132),$J15&gt;=($R$2+126)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="AF15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+139),$J15&gt;=($R$2+133)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="AG15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+146),$J15&gt;=($R$2+140)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="AH15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+153),$J15&gt;=($R$2+147)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="AI15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+160),$J15&gt;=($R$2+154)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="AJ15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+167),$J15&gt;=($R$2+161)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="AK15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+174),$J15&gt;=($R$2+168)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+      <c r="AL15" s="67">
+        <f>IF(AND($I15&lt;=($R$2+181),$J15&gt;=($R$2+175)),IF($R$4=1,1,IF($R$4=2,$G15,$F15)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="59" t="inlineStr">
+        <is>
+          <t>CV-10</t>
+        </is>
+      </c>
+      <c r="B16" s="60" t="inlineStr">
+        <is>
+          <t>Bê tông cống đôi 2x(3x3) phân đoạn 3</t>
+        </is>
+      </c>
+      <c r="C16" s="61" t="n">
+        <v>4200</v>
+      </c>
+      <c r="D16" s="59" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E16" s="61" t="n">
+        <v>93.33</v>
+      </c>
+      <c r="F16" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="59" t="n">
+        <v>14</v>
+      </c>
+      <c r="H16" s="62" t="n">
+        <v>45</v>
+      </c>
+      <c r="I16" s="63">
+        <f>J15+1</f>
+        <v/>
+      </c>
+      <c r="J16" s="64">
+        <f>I16+H16-1</f>
+        <v/>
+      </c>
+      <c r="K16" s="65" t="inlineStr">
+        <is>
+          <t>CV-09</t>
+        </is>
+      </c>
+      <c r="L16" s="66" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="M16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+6),$J16&gt;=($R$2+0)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="N16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+13),$J16&gt;=($R$2+7)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="O16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+20),$J16&gt;=($R$2+14)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="P16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+27),$J16&gt;=($R$2+21)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="Q16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+34),$J16&gt;=($R$2+28)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="R16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+41),$J16&gt;=($R$2+35)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="S16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+48),$J16&gt;=($R$2+42)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="T16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+55),$J16&gt;=($R$2+49)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="U16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+62),$J16&gt;=($R$2+56)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="V16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+69),$J16&gt;=($R$2+63)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="W16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+76),$J16&gt;=($R$2+70)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="X16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+83),$J16&gt;=($R$2+77)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="Y16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+90),$J16&gt;=($R$2+84)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="Z16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+97),$J16&gt;=($R$2+91)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="AA16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+104),$J16&gt;=($R$2+98)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="AB16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+111),$J16&gt;=($R$2+105)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="AC16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+118),$J16&gt;=($R$2+112)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="AD16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+125),$J16&gt;=($R$2+119)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="AE16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+132),$J16&gt;=($R$2+126)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="AF16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+139),$J16&gt;=($R$2+133)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="AG16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+146),$J16&gt;=($R$2+140)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="AH16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+153),$J16&gt;=($R$2+147)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="AI16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+160),$J16&gt;=($R$2+154)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="AJ16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+167),$J16&gt;=($R$2+161)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="AK16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+174),$J16&gt;=($R$2+168)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+      <c r="AL16" s="67">
+        <f>IF(AND($I16&lt;=($R$2+181),$J16&gt;=($R$2+175)),IF($R$4=1,1,IF($R$4=2,$G16,$F16)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="65" t="inlineStr">
+        <is>
+          <t>CV-11</t>
+        </is>
+      </c>
+      <c r="B17" s="69" t="inlineStr">
+        <is>
+          <t>Chống thấm, chèn khe co giãn bitum &amp; Lấp đất</t>
+        </is>
+      </c>
+      <c r="C17" s="70" t="n">
+        <v>11081.91</v>
+      </c>
+      <c r="D17" s="65" t="inlineStr">
+        <is>
+          <t>m3</t>
+        </is>
+      </c>
+      <c r="E17" s="70" t="n">
+        <v>738.79</v>
+      </c>
+      <c r="F17" s="65" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="65" t="n">
+        <v>6</v>
+      </c>
+      <c r="H17" s="71" t="n">
+        <v>15</v>
+      </c>
+      <c r="I17" s="72">
+        <f>J16+1</f>
+        <v/>
+      </c>
+      <c r="J17" s="72">
+        <f>I17+H17-1</f>
+        <v/>
+      </c>
+      <c r="K17" s="65" t="inlineStr">
+        <is>
+          <t>CV-10</t>
+        </is>
+      </c>
+      <c r="L17" s="66" t="inlineStr">
+        <is>
+          <t>CRITICAL</t>
+        </is>
+      </c>
+      <c r="M17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+6),$J17&gt;=($R$2+0)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="N17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+13),$J17&gt;=($R$2+7)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="O17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+20),$J17&gt;=($R$2+14)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="P17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+27),$J17&gt;=($R$2+21)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="Q17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+34),$J17&gt;=($R$2+28)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="R17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+41),$J17&gt;=($R$2+35)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="S17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+48),$J17&gt;=($R$2+42)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="T17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+55),$J17&gt;=($R$2+49)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="U17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+62),$J17&gt;=($R$2+56)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="V17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+69),$J17&gt;=($R$2+63)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="W17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+76),$J17&gt;=($R$2+70)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="X17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+83),$J17&gt;=($R$2+77)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="Y17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+90),$J17&gt;=($R$2+84)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="Z17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+97),$J17&gt;=($R$2+91)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="AA17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+104),$J17&gt;=($R$2+98)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="AB17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+111),$J17&gt;=($R$2+105)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="AC17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+118),$J17&gt;=($R$2+112)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="AD17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+125),$J17&gt;=($R$2+119)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="AE17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+132),$J17&gt;=($R$2+126)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="AF17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+139),$J17&gt;=($R$2+133)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="AG17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+146),$J17&gt;=($R$2+140)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="AH17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+153),$J17&gt;=($R$2+147)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="AI17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+160),$J17&gt;=($R$2+154)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="AJ17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+167),$J17&gt;=($R$2+161)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="AK17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+174),$J17&gt;=($R$2+168)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+      <c r="AL17" s="67">
+        <f>IF(AND($I17&lt;=($R$2+181),$J17&gt;=($R$2+175)),IF($R$4=1,1,IF($R$4=2,$G17,$F17)),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="65" t="inlineStr">
+        <is>
+          <t>CV-12</t>
+        </is>
+      </c>
+      <c r="B18" s="69" t="inlineStr">
+        <is>
+          <t>Nghiệm thu hoàn thành &amp; Bàn giao thông tuyến</t>
+        </is>
+      </c>
+      <c r="C18" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="D18" s="65" t="inlineStr">
+        <is>
+          <t>hồ sơ</t>
+        </is>
+      </c>
+      <c r="E18" s="70" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F18" s="65" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="65" t="n">
+        <v>8</v>
+      </c>
+      <c r="H18" s="71" t="n">
         <v>5</v>
       </c>
-      <c r="H6" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="32" t="inlineStr">
+      <c r="I18" s="72">
+        <f>J17+1</f>
+        <v/>
+      </c>
+      <c r="J18" s="72">
+        <f>I18+H18-1</f>
+        <v/>
+      </c>
+      <c r="K18" s="65" t="inlineStr">
+        <is>
+          <t>CV-11</t>
+        </is>
+      </c>
+      <c r="L18" s="66" t="inlineStr">
         <is>
           <t>CRITICAL</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>CV-03</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>Đóng cọc tre &amp; Đệm cát đầu cọc phân đoạn 1</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>CV-02</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="H7" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="32" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>CV-04</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Bê tông lót móng M100 phân đoạn 1</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>CV-03</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>35</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>35</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="32" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>CV-05</t>
-        </is>
-      </c>
-      <c r="B9" s="8" t="inlineStr">
-        <is>
-          <t>Gia công lắp dựng cốt thép &amp; ván khuôn cống 2x2</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>CV-04</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>35</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>55</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>35</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>55</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="32" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>CV-06</t>
-        </is>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>Đổ bê tông thân cống B20 &amp; Bảo dưỡng</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>CV-05</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>55</v>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>65</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>55</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>65</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J10" s="32" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>CV-07</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="inlineStr">
-        <is>
-          <t>Đào hố móng phân đoạn 2 (Cống 3x3)</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>CV-02</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>25</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>45</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>NON-CRITICAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>CV-08</t>
-        </is>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Đổ bê tông thân cống 3x3 phân đoạn 2</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>30</v>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>CV-07</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>40</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>70</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>45</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>75</v>
-      </c>
-      <c r="I12" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>NON-CRITICAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>CV-09</t>
-        </is>
-      </c>
-      <c r="B13" s="8" t="inlineStr">
-        <is>
-          <t>Đào móng phân đoạn 3 (Cống đôi 2x(3x3))</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="n">
-        <v>35</v>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>CV-06</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="n">
-        <v>65</v>
-      </c>
-      <c r="F13" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="G13" s="4" t="n">
-        <v>65</v>
-      </c>
-      <c r="H13" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="I13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="32" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="20" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>CV-10</t>
-        </is>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Bê tông cống đôi 2x(3x3) phân đoạn 3</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>45</v>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>CV-09</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>145</v>
-      </c>
-      <c r="G14" s="4" t="n">
-        <v>100</v>
-      </c>
-      <c r="H14" s="4" t="n">
-        <v>145</v>
-      </c>
-      <c r="I14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="32" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>CV-11</t>
-        </is>
-      </c>
-      <c r="B15" s="8" t="inlineStr">
-        <is>
-          <t>Chống thấm, chèn khe co giãn bitum &amp; Lấp đất</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="n">
-        <v>15</v>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>CV-10</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="n">
-        <v>145</v>
-      </c>
-      <c r="F15" s="4" t="n">
-        <v>160</v>
-      </c>
-      <c r="G15" s="4" t="n">
-        <v>145</v>
-      </c>
-      <c r="H15" s="4" t="n">
-        <v>160</v>
-      </c>
-      <c r="I15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="32" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>CV-12</t>
-        </is>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Nghiệm thu hoàn thành &amp; Bàn giao thông tuyến</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>CV-11</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>160</v>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>165</v>
-      </c>
-      <c r="G16" s="4" t="n">
-        <v>160</v>
-      </c>
-      <c r="H16" s="4" t="n">
-        <v>165</v>
-      </c>
-      <c r="I16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="32" t="inlineStr">
-        <is>
-          <t>CRITICAL</t>
-        </is>
+      <c r="M18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+6),$J18&gt;=($R$2+0)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="N18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+13),$J18&gt;=($R$2+7)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="O18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+20),$J18&gt;=($R$2+14)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="P18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+27),$J18&gt;=($R$2+21)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="Q18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+34),$J18&gt;=($R$2+28)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="R18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+41),$J18&gt;=($R$2+35)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="S18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+48),$J18&gt;=($R$2+42)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="T18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+55),$J18&gt;=($R$2+49)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="U18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+62),$J18&gt;=($R$2+56)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="V18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+69),$J18&gt;=($R$2+63)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="W18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+76),$J18&gt;=($R$2+70)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="X18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+83),$J18&gt;=($R$2+77)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="Y18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+90),$J18&gt;=($R$2+84)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="Z18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+97),$J18&gt;=($R$2+91)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="AA18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+104),$J18&gt;=($R$2+98)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="AB18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+111),$J18&gt;=($R$2+105)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="AC18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+118),$J18&gt;=($R$2+112)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="AD18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+125),$J18&gt;=($R$2+119)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="AE18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+132),$J18&gt;=($R$2+126)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="AF18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+139),$J18&gt;=($R$2+133)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="AG18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+146),$J18&gt;=($R$2+140)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="AH18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+153),$J18&gt;=($R$2+147)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="AI18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+160),$J18&gt;=($R$2+154)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="AJ18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+167),$J18&gt;=($R$2+161)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="AK18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+174),$J18&gt;=($R$2+168)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
+      </c>
+      <c r="AL18" s="67">
+        <f>IF(AND($I18&lt;=($R$2+181),$J18&gt;=($R$2+175)),IF($R$4=1,1,IF($R$4=2,$G18,$F18)),"")</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <conditionalFormatting sqref="M7:AL18">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>M7&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>